<commit_message>
clean repo and add gitignore
</commit_message>
<xml_diff>
--- a/backend/data/sample_input.xlsx
+++ b/backend/data/sample_input.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhaowenqi/Desktop/ai_supply_chain_planner/backend/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{59140E4A-41F5-8748-9C96-5D34AC45DA43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CD1EAE9-87F5-274E-A595-3970701B2096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16300" activeTab="3" xr2:uid="{D4E04EF5-5C5C-A649-A83B-B67B0DAD4C19}"/>
+    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16260" activeTab="2" xr2:uid="{D4E04EF5-5C5C-A649-A83B-B67B0DAD4C19}"/>
   </bookViews>
   <sheets>
     <sheet name="ProductionPlan" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="11">
   <si>
     <t>date</t>
   </si>
@@ -65,16 +65,23 @@
     <t>MAT_002</t>
   </si>
   <si>
-    <t>supply</t>
-  </si>
-  <si>
-    <t>opening_stock</t>
+    <t>SKU_B</t>
+  </si>
+  <si>
+    <t>MAT_003</t>
+  </si>
+  <si>
+    <t>qty</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <sz val="12"/>
@@ -123,7 +130,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -133,6 +140,8 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -467,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C446928-295E-BE47-981B-5CCD01166F0B}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -482,25 +491,157 @@
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="2">
+      <c r="A2" s="3">
         <v>46113</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C2">
-        <v>100</v>
+      <c r="C2" s="4">
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="2">
+      <c r="A3" s="3">
         <v>46114</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C3">
-        <v>120</v>
+      <c r="C3" s="4">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="3">
+        <v>46115</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="4">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="3">
+        <v>46116</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="4">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="3">
+        <v>46117</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="4">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="3">
+        <v>46118</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" s="4">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="3">
+        <v>46119</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="4">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="3">
+        <v>46113</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="3">
+        <v>46114</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="4">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="3">
+        <v>46115</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="3">
+        <v>46116</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" s="4">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="3">
+        <v>46117</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="3">
+        <v>46118</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="4">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="3">
+        <v>46119</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="4">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -511,7 +652,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D74713F-6EA6-C24D-B355-B5DFAF1BC598}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -526,25 +667,47 @@
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" t="s">
+      <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="4">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" t="s">
+      <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="4">
         <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="4">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -555,7 +718,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E90B60CC-10FB-5148-9043-1607434C6D0D}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -566,29 +729,128 @@
         <v>4</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="2">
+      <c r="A2" s="3">
         <v>46113</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="4">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="3">
+        <v>46115</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="4">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="3">
+        <v>46117</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="4">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="3">
+        <v>46119</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="4">
         <v>120</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="2">
+    <row r="6" spans="1:3">
+      <c r="A6" s="3">
         <v>46114</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C3">
-        <v>80</v>
+      <c r="C6" s="4">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="3">
+        <v>46116</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="4">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="3">
+        <v>46118</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="4">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="3">
+        <v>46113</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="4">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="3">
+        <v>46115</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="4">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="3">
+        <v>46117</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="4">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="3">
+        <v>46119</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="4">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -599,32 +861,62 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41A81C73-000E-144B-BE63-7AC04EBCD758}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="1"/>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="4">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="4">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="4" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3">
-        <v>300</v>
-      </c>
+      <c r="B4" s="4">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="2"/>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="2"/>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="2"/>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="2"/>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="2"/>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="2"/>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>